<commit_message>
chore: crawl 2026-08-05 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore: crawl 2026-08-08 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G199"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3538,14 +3538,14 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
+          <t>Edital Conjunto nº 6/2026 - CAPES/CNJ - Apoio a Pesquisas Judiciárias, formato, pdf, 257kb</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2873621_sei___23038-001405_2026_81.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F109" t="n">
@@ -3561,24 +3561,20 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>3</v>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3588,22 +3584,22 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
+          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3615,22 +3611,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3642,22 +3638,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
+          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3669,22 +3665,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
+          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3696,22 +3692,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
+          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3723,22 +3719,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
+          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3750,20 +3746,24 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>1</v>
-      </c>
-      <c r="G117" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3773,24 +3773,20 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
+          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>2</v>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3800,20 +3796,24 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
+          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>1</v>
-      </c>
-      <c r="G119" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3823,14 +3823,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
+          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -3846,14 +3846,14 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
+          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F121" t="n">
@@ -3869,24 +3869,20 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
+          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>3</v>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3896,20 +3892,24 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
+          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>1</v>
-      </c>
-      <c r="G123" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3919,24 +3919,20 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
+          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F124" t="n">
-        <v>2</v>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3946,14 +3942,14 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
+          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F125" t="n">
@@ -3961,7 +3957,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3973,20 +3969,24 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
+          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>1</v>
-      </c>
-      <c r="G126" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3996,24 +3996,20 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
+          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>3</v>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4023,14 +4019,14 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
+          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F128" t="n">
@@ -4038,7 +4034,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
+          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4050,22 +4046,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
+          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4077,22 +4073,22 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
+          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F130" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
+          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4104,14 +4100,14 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
+          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F131" t="n">
@@ -4119,7 +4115,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
+          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4131,14 +4127,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
+          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -4146,7 +4142,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4158,22 +4154,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
+          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4185,20 +4181,24 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
+          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>1</v>
-      </c>
-      <c r="G134" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4208,14 +4208,14 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
+          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F135" t="n">
@@ -4231,24 +4231,20 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
+          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>3</v>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4258,22 +4254,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4285,20 +4281,24 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
+          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>1</v>
-      </c>
-      <c r="G138" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4308,24 +4308,20 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
+          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>2</v>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4335,14 +4331,14 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
+          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
         </is>
       </c>
       <c r="F140" t="n">
@@ -4350,7 +4346,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4362,20 +4358,24 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
+          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F141" t="n">
-        <v>1</v>
-      </c>
-      <c r="G141" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4385,14 +4385,14 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
+          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F142" t="n">
@@ -4408,24 +4408,20 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
+          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>4</v>
-      </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4435,14 +4431,14 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
+          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F144" t="n">
@@ -4450,7 +4446,7 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4462,14 +4458,14 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
+          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F145" t="n">
@@ -4477,7 +4473,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
+          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4489,14 +4485,14 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
+          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F146" t="n">
@@ -4504,7 +4500,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
+          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4516,22 +4512,22 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
+          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4543,37 +4539,41 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
+          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F148" t="n">
-        <v>1</v>
-      </c>
-      <c r="G148" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
+          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F149" t="n">
@@ -4589,14 +4589,14 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F150" t="n">
@@ -4612,14 +4612,14 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
+          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
         </is>
       </c>
       <c r="F151" t="n">
@@ -4635,14 +4635,14 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
+          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
         </is>
       </c>
       <c r="F152" t="n">
@@ -4658,14 +4658,14 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
+          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
         </is>
       </c>
       <c r="F153" t="n">
@@ -4681,14 +4681,14 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
+          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
         </is>
       </c>
       <c r="F154" t="n">
@@ -4704,14 +4704,14 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
+          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
         </is>
       </c>
       <c r="F155" t="n">
@@ -4727,14 +4727,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
+          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -4750,14 +4750,14 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
+          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -4773,14 +4773,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
+          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -4796,14 +4796,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
+          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -4819,14 +4819,14 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -4842,14 +4842,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
+          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -4865,14 +4865,14 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
+          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -4888,14 +4888,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
+          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -4911,14 +4911,14 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
+          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -4934,14 +4934,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
+          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -4957,14 +4957,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
+          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -4980,14 +4980,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
+          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -5003,14 +5003,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -5026,14 +5026,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
+          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -5049,14 +5049,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
+          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -5072,14 +5072,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -5095,14 +5095,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
+          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -5118,14 +5118,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Edital nº 26 versão consolidada</t>
+          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -5141,14 +5141,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 26 versão consolidada</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -5164,24 +5164,20 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
+          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
         </is>
       </c>
       <c r="F175" t="n">
-        <v>2</v>
-      </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5191,20 +5187,24 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
+          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
         </is>
       </c>
       <c r="F176" t="n">
-        <v>1</v>
-      </c>
-      <c r="G176" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5214,14 +5214,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
+          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -5237,14 +5237,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
+          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -5260,14 +5260,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
+          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -5283,14 +5283,14 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -5306,14 +5306,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
+          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -5329,14 +5329,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
+          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -5352,14 +5352,14 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
+          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -5375,14 +5375,14 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
+          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -5398,14 +5398,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
+          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -5421,14 +5421,14 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
+          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -5444,14 +5444,14 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -5467,14 +5467,14 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
+          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -5490,14 +5490,14 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
+          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -5513,14 +5513,14 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -5536,14 +5536,14 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
+          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -5559,14 +5559,14 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
+          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -5582,14 +5582,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
+          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -5605,14 +5605,14 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -5628,14 +5628,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -5651,24 +5651,20 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
         </is>
       </c>
       <c r="F196" t="n">
-        <v>2</v>
-      </c>
-      <c r="G196" t="inlineStr">
-        <is>
-          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -5678,20 +5674,24 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
         </is>
       </c>
       <c r="F197" t="n">
-        <v>1</v>
-      </c>
-      <c r="G197" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -5701,14 +5701,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -5724,20 +5724,43 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>1</v>
+      </c>
+      <c r="G199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr"/>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr">
+        <is>
           <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/2147-resultado-preliminar.pdf</t>
         </is>
       </c>
-      <c r="F199" t="n">
-        <v>1</v>
-      </c>
-      <c r="G199" t="inlineStr"/>
+      <c r="F200" t="n">
+        <v>1</v>
+      </c>
+      <c r="G200" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: crawl 2026-08-14 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -511,9 +511,13 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Chamada Pública CNPq/ERC (Conselho Europeu de Pesquisa) Nº 21/2026 | https://www.gov.br/cnpq/pt-br/chamadas/todas-as-chamadas/chamadas-2026/chamada-no-21-2026/chamada-publica-cnpq-N-21-2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3526,9 +3530,13 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>1</v>
-      </c>
-      <c r="G108" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Edital Conjunto nº 5/2026 - Programa OBEDUC-EI, formato, pdf, 9,67mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital-no-5.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4007,9 +4015,13 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>1</v>
-      </c>
-      <c r="G127" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">

</xml_diff>

<commit_message>
chore: crawl 2026-08-15 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1560,11 +1560,11 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Alteração do edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato - pdf, 60,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11052026_Edital_2817202_SEI_2816655_Edital_n__26_2025___Alteracao.pdf</t>
+          <t>Edital nº 26/2025 - Alteração, formato, pdf, 114kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878184_edital_26_2025___alteracao.pdf/@@display-file/file ; Alteração do edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato - pdf, 60,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11052026_Edital_2817202_SEI_2816655_Edital_n__26_2025___Alteracao.pdf</t>
         </is>
       </c>
     </row>
@@ -3569,20 +3569,24 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
+          <t>Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 87kb</t>
         </is>
       </c>
       <c r="C110" t="inlineStr"/>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/26022024_Edital_2328837_SEI_2326326_Edital_02_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1</v>
-      </c>
-      <c r="G110" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 02/2024 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16052024_Edital_2379426_SEI_2379169_Edital_02_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3592,24 +3596,20 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 039/2013 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 400kb</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_039_2013_PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F111" t="n">
-        <v>3</v>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3619,22 +3619,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
+          <t>Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933938_Edital_5_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F112" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 60kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400239_SEI_2399449_Edital_05_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 05/2023 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984677_Lista_de_inscritos_Math_Amsud_Edital_5.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3646,22 +3646,22 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 239kb</t>
         </is>
       </c>
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
+          <t>Edital nº 05/2024 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file ; Alteração do Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373417_SEI_2372656_Edital_05_2024.pdf/@@display-file/file ; Edital nº 05/2024 - ProgramaCAPES/MATH-AMSUD, formato - pdf, 239kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20032024_Edital_2343766_SEI_2342530_Edital_05_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3673,22 +3673,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
+          <t>Edital nº 06/2023 - ProgramaCAPES/STIC-AMSUD, formato - pdf, 473kb</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933950_Edital_6_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F114" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400119_SEI_2399429_Edital_6_2023___Alteracao_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 06/2023 - Programa CAPES/STIC-AMSUD, formato - pdf, 571kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984493_Lista_de_inscritos_Stic_Amsud_Edital_6.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3700,22 +3700,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
+          <t>Edital nº 06/2024 - PDSE - formato, pdf, 133kb</t>
         </is>
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21032024_Edital_2344636_SEI_2343579_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 06/2024 - PDSE - formato, pdf, 55kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10052024_Edital_2376323_SEI_2375557_Edital_6_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3727,22 +3727,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
+          <t>Edital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 466kb</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15032023_Edital_1933965_Edital_7_2023_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 07/2023 - ProgramaCAPES/CLIMAT-AMSUD, formato - pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400133_SEI_2399445_Edital_07_2023___ALTERACAO_II.pdf/@@display-file/file ; Relação das inscrições do Edital nº 07/2023 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 570kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/30052023_Lista_Listagem_1984693_Lista_de_inscritos_Climat_Amsud_Edital_7.2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3754,22 +3754,22 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
+          <t>Edital nº 08/2023 - CAPES/Cofecub, formato, pdf, 495kb</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03042023_Edital_1946708_Edital_8_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F117" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+          <t>Alteração doEdital nº 08/2023 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20062024_Edital_2401059_SEI_2399441_Edital_08_2023___ALTERACAO_II.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3781,20 +3781,24 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 213kb</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22032024_Edital_2345736_SEI_2343959_Edital_8.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F118" t="n">
-        <v>1</v>
-      </c>
-      <c r="G118" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 08/2024 - Programa CAPES/Cofecub, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23122024_Edital_2517712_SEI_2516934_Edital_8_2024.pdf/@@display-file/file ; Prorrogação do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02072024_Edital_2409554_SEI_2409272_Edital_08_2024___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 08/2024 - CAPES/Cofecub, formato, pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07052024_Edital_2373782_SEI_2372654_Edital_08_2024.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3804,24 +3808,20 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
+          <t>Edital nº 10/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16022022_Edital10.22PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>2</v>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3831,14 +3831,14 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
+          <t>Edital nº 14/2025 - PCI - pdf, 83kb</t>
         </is>
       </c>
       <c r="C120" t="inlineStr"/>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31072025_Edital_2646654_SEI_2644987_Edital_14_2025.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F120" t="n">
@@ -3854,20 +3854,24 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
+          <t>Edital nº 16/2025 - formato, pdf, 360kb</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11082025_Edital_2654124.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F121" t="n">
-        <v>1</v>
-      </c>
-      <c r="G121" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Lista de inscritos no edital nº 16/2025 - formato, pdf, 207kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2693783_SEI___23038.003238_2025_21_buffalo.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3877,14 +3881,14 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
+          <t>Edital nº 16/2026 - Programa AURORA — Continuidade da Trajetória de Mães Cientistas</t>
         </is>
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2818271_SEI_2817084_Edital_16_2026__1_.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F122" t="n">
@@ -3900,24 +3904,20 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
+          <t>Edital nº 19/2017 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 315kb</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/31052017Edital192017PDPI.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F123" t="n">
-        <v>3</v>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3927,14 +3927,14 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
+          <t>Edital nº 19/2026 - Programa Capes/Universidade em Buffalo (Capes/UB) - Professor Visitante - formato, pdf, 139kb</t>
         </is>
       </c>
       <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr"/>
       <c r="E124" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2843097_SEI_2842333_Edital_n__19_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F124" t="n">
@@ -3950,22 +3950,22 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
+          <t>Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 286kb</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
       <c r="D125" t="inlineStr"/>
       <c r="E125" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07042022_Edital_1673688_EDITAL_20_2022_STIC_AMSUD.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 20/2022 -Programa CAPES/STIC-AMSUD, formato, pdf - 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400177_SEI_2399435_Edital_20_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 20/2022 - Programa CAPES/STIC-AMSUD, formato - pdf, 358kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727082_STIC.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -3977,22 +3977,22 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
+          <t>Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 281kb</t>
         </is>
       </c>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="inlineStr"/>
       <c r="E126" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24082023_Edital_2043434_Edital_21_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F126" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Retificação do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/01112023_Edital_2262651_SEI_2262236_Edital_21_2023.pdf/@@display-file/file ; Alteração do Edital nº 21/2023 - Projetos de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/31102023_Edital_2261925_SEI_2261451_Edital_22_2023.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4004,24 +4004,20 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
+          <t>Edital nº 21/2026 - Programa de Desenvolvimento da Pós-Graduação (PDPG) – Parcerias Estratégicas nos Estados VI – Rede de Pesquisa e Desenvolvimento da Região Nordeste, formato, pdf, 177kb</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="inlineStr"/>
       <c r="E127" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2848691_sei_2847430_edital_n__21_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F127" t="n">
-        <v>2</v>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4031,22 +4027,22 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
+          <t>Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 150kb</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/sei_2849220_edital_n__22_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F128" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 22/2026 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 47,4kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2858430_sei_2857160_edital_22_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4058,22 +4054,22 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
+          <t>Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2851776_sei_2851450_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F129" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4085,14 +4081,14 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
+          <t>Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 168kb</t>
         </is>
       </c>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855421_sei_2854365_edital_n__23_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F130" t="n">
@@ -4100,7 +4096,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 23/2026 - Programa Nacional de Formação de Professores da Educação Básica (PARFOR), formato, pdf, 130kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2875930_edital_23_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4112,24 +4108,20 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
+          <t>Edital nº 24/2026 - Cooperação entre Instituições para</t>
         </is>
       </c>
       <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878169_edital_24_2026___pci.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F131" t="n">
-        <v>3</v>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4139,14 +4131,14 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
+          <t>Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04052022_Edital_1698011_SEI_CAPES___1696119___Edital_25.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F132" t="n">
@@ -4154,7 +4146,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
+          <t>Alteração do edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 67kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400217_SEI_2399433_Edital_25_2022___ALTERACAO_I.pdf/@@display-file/file ; Relação das inscrições do Edital nº 25/2022 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 353kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06062022_Lista_Listagem_1727108_Climat.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4166,22 +4158,22 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
+          <t>Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 83kb</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
       <c r="D133" t="inlineStr"/>
       <c r="E133" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/17092024_Edital_2461148_SEI_2460992_Edital_25_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F133" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 25/2024 - Chamada Pública para envio de Proposta de Projeto de Cooperação entre Instituições para Qualificação de Profissionais de Nível Superior (PCI) - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10122024_Edital_2510251_SEI_2508924_Edital_25_2024___Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4193,22 +4185,22 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
+          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
         </is>
       </c>
       <c r="C134" t="inlineStr"/>
       <c r="D134" t="inlineStr"/>
       <c r="E134" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4220,20 +4212,24 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
+          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="inlineStr"/>
       <c r="E135" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F135" t="n">
-        <v>1</v>
-      </c>
-      <c r="G135" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4243,20 +4239,24 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
+          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>1</v>
-      </c>
-      <c r="G136" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4266,14 +4266,14 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
+          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F137" t="n">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4293,22 +4293,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4320,20 +4320,24 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
+          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>1</v>
-      </c>
-      <c r="G139" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4343,24 +4347,20 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
+          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F140" t="n">
-        <v>2</v>
-      </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4370,24 +4370,20 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
+          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F141" t="n">
-        <v>2</v>
-      </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4397,20 +4393,24 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
+          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>1</v>
-      </c>
-      <c r="G142" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4420,20 +4420,24 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
+          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>1</v>
-      </c>
-      <c r="G143" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4443,24 +4447,20 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
+          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F144" t="n">
-        <v>4</v>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4470,22 +4470,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
+          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
         </is>
       </c>
       <c r="F145" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4497,22 +4497,22 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
+          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F146" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4524,24 +4524,20 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
+          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F147" t="n">
-        <v>4</v>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4551,24 +4547,20 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
+          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F148" t="n">
-        <v>3</v>
-      </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4578,129 +4570,149 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
+          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F149" t="n">
-        <v>1</v>
-      </c>
-      <c r="G149" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
+          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F150" t="n">
-        <v>1</v>
-      </c>
-      <c r="G150" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
+          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F151" t="n">
-        <v>1</v>
-      </c>
-      <c r="G151" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
+          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F152" t="n">
-        <v>1</v>
-      </c>
-      <c r="G152" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
+          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F153" t="n">
-        <v>1</v>
-      </c>
-      <c r="G153" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
+          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F154" t="n">
@@ -4716,14 +4728,14 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F155" t="n">
@@ -4739,14 +4751,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
+          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -4762,14 +4774,14 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
+          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
         </is>
       </c>
       <c r="F157" t="n">
@@ -4785,14 +4797,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
+          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -4808,14 +4820,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
+          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -4831,14 +4843,14 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
+          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -4854,14 +4866,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -4877,14 +4889,14 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
+          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -4900,14 +4912,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
+          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -4923,14 +4935,14 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
+          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -4946,14 +4958,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
+          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -4969,14 +4981,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
+          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -4992,14 +5004,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
+          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -5015,14 +5027,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
+          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -5038,14 +5050,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -5061,14 +5073,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
+          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -5084,14 +5096,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
+          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -5107,14 +5119,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -5130,14 +5142,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
+          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -5153,14 +5165,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Edital nº 26 versão consolidada</t>
+          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -5176,14 +5188,14 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -5199,24 +5211,20 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
+          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
         </is>
       </c>
       <c r="F176" t="n">
-        <v>2</v>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -5226,14 +5234,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
+          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -5249,14 +5257,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
+          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -5272,14 +5280,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
+          <t>Edital nº 26 versão consolidada</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -5295,14 +5303,14 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
+          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -5318,20 +5326,24 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
         </is>
       </c>
       <c r="F181" t="n">
-        <v>1</v>
-      </c>
-      <c r="G181" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -5341,14 +5353,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
+          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -5364,14 +5376,14 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
+          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -5387,14 +5399,14 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
+          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
         </is>
       </c>
       <c r="F184" t="n">
@@ -5410,14 +5422,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
+          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -5433,14 +5445,14 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
+          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -5456,14 +5468,14 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
+          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -5479,14 +5491,14 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -5502,14 +5514,14 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
+          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -5525,14 +5537,14 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
+          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -5548,14 +5560,14 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -5571,14 +5583,14 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
+          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -5594,14 +5606,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
+          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -5617,14 +5629,14 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
+          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -5640,14 +5652,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -5663,14 +5675,14 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -5686,24 +5698,20 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
         </is>
       </c>
       <c r="F197" t="n">
-        <v>2</v>
-      </c>
-      <c r="G197" t="inlineStr">
-        <is>
-          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -5713,14 +5721,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -5736,14 +5744,14 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -5759,20 +5767,139 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr">
         <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>1</v>
+      </c>
+      <c r="G200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr"/>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>1</v>
+      </c>
+      <c r="G201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr"/>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>2</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr"/>
+      <c r="D203" t="inlineStr"/>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>1</v>
+      </c>
+      <c r="G203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr"/>
+      <c r="D204" t="inlineStr"/>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>1</v>
+      </c>
+      <c r="G204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr"/>
+      <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr">
+        <is>
           <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/2147-resultado-preliminar.pdf</t>
         </is>
       </c>
-      <c r="F200" t="n">
-        <v>1</v>
-      </c>
-      <c r="G200" t="inlineStr"/>
+      <c r="F205" t="n">
+        <v>1</v>
+      </c>
+      <c r="G205" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: crawl 2026-08-19 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -1560,11 +1560,11 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Edital nº 26/2025 - Alteração, formato, pdf, 114kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878184_edital_26_2025___alteracao.pdf/@@display-file/file ; Alteração do edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato - pdf, 60,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11052026_Edital_2817202_SEI_2816655_Edital_n__26_2025___Alteracao.pdf</t>
+          <t>Edital nº 26/2025 - Alteração, formato, pdf, 114kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2878184_edital_26_2025___alteracao.pdf/@@display-file/file ; Retificação_Edital nº 26/2025 - Alteração, formato, pdf, 115kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2879083_edital_26_2025___retificacao.pdf/@@display-file/file ; Alteração do edital nº 26/2025 - Política de Novação para Bolsistas e Ex-Bolsistas no Exterior, formato - pdf, 60,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11052026_Edital_2817202_SEI_2816655_Edital_n__26_2025___Alteracao.pdf</t>
         </is>
       </c>
     </row>
@@ -1854,11 +1854,11 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Prorrogação Edital Conjunto nº 1/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 65,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855428_sei_2855023_edital_conjunto_n__1_2026___prorrogacao.pdf/@@display-file/file ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Angola e México, formato pdf, 435kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/01042026_Lista_Listagem_2788855_Lista_de_inscritos_Angola_e_Mexico.pdf/@@display-file/file ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 421kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/12032026_Lista_Listagem_2780399_Lista_de_Inscritos_Panama.pdf/@@display-file/file ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México - Retificação do Cumprimento de decisão judicial, formato pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13022026_Edital_2768872_SEI_2768349_Edital_Conjunto_n__1_2026____Retificacao_de_Decisao_Judicial.pdf/@@display-file/file ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México - Cumprimento de decisão judicial, formato pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11022026_Edital_2766993_SEI_2766572_Edital_Conjunto_1_2026_.pdf/@@display-file/file ; Alteração do edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 81kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03022026_Edital_2762271_SEI_2757276_Edital_Conjunto_n__1_2026_CAPES_MIR_____1_.pdf/@@display-file/file ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 151kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09012026_Edital_2748950_SEI_2748603_Edital_Conjunto_n__1_2026.pdf/@@display-file/file ; Alteração do edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México, formato pdf, 81kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03022026_Edital_2762271_SEI_2757276_Edital_Conjunto_n__1_2026_CAPES_MIR_____1_.pdf ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México - Cumprimento de decisão judicial, formato pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11022026_Edital_2766993_SEI_2766572_Edital_Conjunto_1_2026_.pdf ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México - Retificação do Cumprimento de decisão judicial, formato pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13022026_Edital_2768872_SEI_2768349_Edital_Conjunto_n__1_2026____Retificacao_de_Decisao_Judicial.pdf ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México, formato pdf, 421kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/12032026_Lista_Listagem_2780399_Lista_de_Inscritos_Panama.pdf ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesAngola e México, formato pdf, 435kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/01042026_Lista_Listagem_2788855_Lista_de_inscritos_Angola_e_Mexico.pdf</t>
+          <t>Prorrogação Edital Conjunto nº 1/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 65,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2855428_sei_2855023_edital_conjunto_n__1_2026___prorrogacao.pdf/@@display-file/file ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Angola e México, formato pdf, 435kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/01042026_Lista_Listagem_2788855_Lista_de_inscritos_Angola_e_Mexico.pdf/@@display-file/file ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 421kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/12032026_Lista_Listagem_2780399_Lista_de_Inscritos_Panama.pdf/@@display-file/file ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México - Retificação do Cumprimento de decisão judicial, formato pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13022026_Edital_2768872_SEI_2768349_Edital_Conjunto_n__1_2026____Retificacao_de_Decisao_Judicial.pdf/@@display-file/file ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México - Cumprimento de decisão judicial, formato pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11022026_Edital_2766993_SEI_2766572_Edital_Conjunto_1_2026_.pdf/@@display-file/file ; Alteração do edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 81kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03022026_Edital_2762271_SEI_2757276_Edital_Conjunto_n__1_2026_CAPES_MIR_____1_.pdf/@@display-file/file ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  Edições Panamá, Angola e México, formato pdf, 151kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09012026_Edital_2748950_SEI_2748603_Edital_Conjunto_n__1_2026.pdf/@@display-file/file ; Edital Conjunto nº 1/2026 - Prorrogação formato, pdf, 113kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2879086_edital_conjunto_1_2026___prorrogacao.pdf/@@display-file/file ; Alteração do edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México, formato pdf, 81kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/03022026_Edital_2762271_SEI_2757276_Edital_Conjunto_n__1_2026_CAPES_MIR_____1_.pdf ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México - Cumprimento de decisão judicial, formato pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11022026_Edital_2766993_SEI_2766572_Edital_Conjunto_1_2026_.pdf ; Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México - Retificação do Cumprimento de decisão judicial, formato pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13022026_Edital_2768872_SEI_2768349_Edital_Conjunto_n__1_2026____Retificacao_de_Decisao_Judicial.pdf ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesPanamá, Angola e México, formato pdf, 421kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/12032026_Lista_Listagem_2780399_Lista_de_Inscritos_Panama.pdf ; Lista de inscritos Edital Conjunto nº 01/2026 - Programa Caminhos Amefricanos: Programa de Intercâmbios Sul-Sul -  EdiçõesAngola e México, formato pdf, 435kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/01042026_Lista_Listagem_2788855_Lista_de_inscritos_Angola_e_Mexico.pdf</t>
         </is>
       </c>
     </row>
@@ -2009,9 +2009,13 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Alteração - Edital nº 6/2026 Programa Rede de Pesquisa e Desenvolvimento da Amazônia Legal - formato, pdf, 125kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2879953_alteracao_edital_6_2026.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">

</xml_diff>

<commit_message>
chore: crawl 2026-08-22 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -4131,11 +4131,11 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file</t>
+          <t>Alteração Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 102kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2872644_edital_conjunto_23_2026___alteracao.pdf/@@display-file/file ; Relação dos Programas de Pós-Graduação (PPGs) - Edital nº 23/2026 - Programa de Desenvolvimento Acadêmico Indígena (PDAI), formato, pdf, 1.836kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/resultado_2881142_pdai_divulgacao_ppgs_bolsas_v-final_13-08-2026.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: crawl 2026-08-25 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G207"/>
+  <dimension ref="A1:G208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4817,14 +4817,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -4840,14 +4840,14 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
+          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
         </is>
       </c>
       <c r="F159" t="n">
@@ -4863,14 +4863,14 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
+          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
         </is>
       </c>
       <c r="F160" t="n">
@@ -4886,14 +4886,14 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
+          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
         </is>
       </c>
       <c r="F161" t="n">
@@ -4909,14 +4909,14 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
+          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -4932,14 +4932,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
+          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -4955,14 +4955,14 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
+          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -4978,14 +4978,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
+          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -5001,14 +5001,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
+          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -5024,14 +5024,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
+          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -5047,14 +5047,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -5070,14 +5070,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
+          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -5093,14 +5093,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
+          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -5116,14 +5116,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
+          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -5139,14 +5139,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
+          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -5162,14 +5162,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
+          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -5185,14 +5185,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
+          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -5208,14 +5208,14 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
+          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -5231,14 +5231,14 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -5254,14 +5254,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
+          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -5277,14 +5277,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
+          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -5300,14 +5300,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -5323,14 +5323,14 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
+          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -5346,14 +5346,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Edital nº 26 versão consolidada</t>
+          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -5369,14 +5369,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 26 versão consolidada</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -5392,24 +5392,20 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
+          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
         </is>
       </c>
       <c r="F183" t="n">
-        <v>2</v>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -5419,20 +5415,24 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
+          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
         </is>
       </c>
       <c r="F184" t="n">
-        <v>1</v>
-      </c>
-      <c r="G184" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5442,14 +5442,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
+          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -5465,14 +5465,14 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
+          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -5488,14 +5488,14 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
+          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -5511,14 +5511,14 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -5534,14 +5534,14 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
+          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -5557,14 +5557,14 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
+          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
         </is>
       </c>
       <c r="F190" t="n">
@@ -5580,14 +5580,14 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
+          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -5603,14 +5603,14 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
+          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -5626,14 +5626,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
+          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -5649,14 +5649,14 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
+          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -5672,14 +5672,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -5695,14 +5695,14 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
+          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -5718,14 +5718,14 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
+          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -5741,14 +5741,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -5764,14 +5764,14 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
+          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -5787,14 +5787,14 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
+          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -5810,14 +5810,14 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
+          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -5833,14 +5833,14 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -5856,14 +5856,14 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
         </is>
       </c>
       <c r="F203" t="n">
@@ -5879,24 +5879,20 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
         </is>
       </c>
       <c r="F204" t="n">
-        <v>2</v>
-      </c>
-      <c r="G204" t="inlineStr">
-        <is>
-          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -5906,20 +5902,24 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr"/>
       <c r="E205" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
         </is>
       </c>
       <c r="F205" t="n">
-        <v>1</v>
-      </c>
-      <c r="G205" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -5929,14 +5929,14 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr"/>
       <c r="E206" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
         </is>
       </c>
       <c r="F206" t="n">
@@ -5952,20 +5952,43 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr">
         <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>1</v>
+      </c>
+      <c r="G207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr"/>
+      <c r="D208" t="inlineStr"/>
+      <c r="E208" t="inlineStr">
+        <is>
           <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/2147-resultado-preliminar.pdf</t>
         </is>
       </c>
-      <c r="F207" t="n">
-        <v>1</v>
-      </c>
-      <c r="G207" t="inlineStr"/>
+      <c r="F208" t="n">
+        <v>1</v>
+      </c>
+      <c r="G208" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: crawl 2026-08-28 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G208"/>
+  <dimension ref="A1:G214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4251,24 +4251,20 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
+          <t>Edital nº 25/2026 - Edição 2027, formato, pdf, 145kb</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="inlineStr"/>
       <c r="E136" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2886643_sei_2886062_edital_n___25_2026.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F136" t="n">
-        <v>3</v>
-      </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4278,22 +4274,22 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
+          <t>Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - Retificação - formato, pdf, 48kb</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="inlineStr"/>
       <c r="E137" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/14102024_Edital_2477735_SEI_2477608_Edital_N__26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F137" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
+          <t>Alteração do Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/13032025_Edital_2560841_SEI_2559847_Edital_26_2024___ALTERACAO.pdf/@@display-file/file ; Edital nº 26/2024 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 135kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102024_Edital_2474014_SEI_2472849_Edital_26_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4305,22 +4301,22 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
+          <t>Edital nº 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 157kb</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="inlineStr"/>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/05112024_Edital_2490387_SEI_2489251_Edital_27_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F138" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
+          <t>Alteração do Edital 27/2024 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa no EUA - PDPI - formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02122024_Edital_2505290_SEI_2504109_Edital_27_2024__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4332,14 +4328,14 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
+          <t>Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 110kb</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="inlineStr"/>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/14022020_Edital_1145537_Edital_SITE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F139" t="n">
@@ -4347,7 +4343,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
+          <t>Reabertura e alteração do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 222kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28042022_Edital_1691552_SEI_CAPES___1685746___Edital_30_2019.pdf/@@display-file/file ; Suspensão do Edital nº 30/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 111kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_1326070_Edital_Suspensao_site.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4359,14 +4355,14 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
+          <t>Edital nº 30/2023 - PDSE - formato, pdf, 125kb</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="inlineStr"/>
       <c r="E140" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/06112023_Edital_2263037_SEI_2261948_Edital_30_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F140" t="n">
@@ -4374,7 +4370,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
+          <t>Prorrogação do Edital nº 30/2023 - PDSE - formato, pdf, 136kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/11012024_Edital_2306448_SEI_CAPES___2305414___Edital_30_2023___Prorrogacao.pdf/@@display-file/file ; Alteração do Edital nº 30/2023 - PDSE - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/18122023_Edital_2293491_SEI_2293429_Edital_30_2023_Alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4386,22 +4382,22 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
+          <t>Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 225kb</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="inlineStr"/>
       <c r="E141" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL32_2022_COFECUB.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F141" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 68kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/19062024_Edital_2400143_SEI_2399437_Edital_32_2022___ALTERACAO_III.pdf/@@display-file/file ; Relação de inscritos do Edital Nº 32/2022 - CAPES/Cofecub, formato, pdf, 65kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/25082022_Lista_Listagem_1783309_EDITAL_32_2022___CAPES_COFECUB_Relacao_de_Inscricoes.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4413,20 +4409,24 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
+          <t>Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 139kb</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="inlineStr"/>
       <c r="E142" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/16112023_Edital_2271416_SEI_2268914_Edital_32_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F142" t="n">
-        <v>1</v>
-      </c>
-      <c r="G142" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 32/2023 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 57kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09022024_SEI_2321458_Edital_N__32_2023___ALTERACAOPDPI.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4436,14 +4436,14 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
+          <t>Edital nº 35/2011 - Certificação em Língua Inglesa - pdf, 615kb</t>
         </is>
       </c>
       <c r="C143" t="inlineStr"/>
       <c r="D143" t="inlineStr"/>
       <c r="E143" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_035_CertificacaoEUAprofLingIngl_Fulbright.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F143" t="n">
@@ -4459,24 +4459,20 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
+          <t>Edital nº 4/2019 - Programa de Desenvolvimento Profissional para Professores de Língua Inglesa nos EUA - PDPI - pdf, 270kb</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="inlineStr"/>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/08022019Edital4.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F144" t="n">
-        <v>3</v>
-      </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4486,22 +4482,22 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
+          <t>Edital nº 44/2012 - Programa de Aperfeiçoamento para Professores de Língua Inglesa nos Eua, pdf, 272kb</t>
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="inlineStr"/>
       <c r="E145" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLingIngl_EUA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+          <t>Edital nº 44/2012 - Retificado - pdf, 528kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_0442012_ProfLIngRetif.pdf/@@display-file/file ; Retificação do Edital nº 44/2012 - pdf, 46kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/RetificacaoEdital442012_ProfLingInglEUA_01out12.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4513,20 +4509,24 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
+          <t>Edital nº 44/2022 - PDSE - formato, pdf, 337kb</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="inlineStr"/>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22122022_Edital_1882688_Edital_44_2022.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F146" t="n">
-        <v>1</v>
-      </c>
-      <c r="G146" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 44/2022 - PDSE - formato, pdf, 146kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23052023_Edital_1981709_Edital_44_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4536,24 +4536,20 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
+          <t>Edital nº 52/2010 - Certificação em Língua Inglesa, pdf, 60kbDF</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Edital_52_Certificacao_LinguaInglesa2010.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F147" t="n">
-        <v>2</v>
-      </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4563,14 +4559,14 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
+          <t>Edital Nº09/2026 - Programa CAPES/BRAFITEC, formato, pdf, 209kb</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="inlineStr"/>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2800035_SEI_2799041_Edital_9__de_2026.pdf</t>
         </is>
       </c>
       <c r="F148" t="n">
@@ -4578,7 +4574,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+          <t>Edital n° 9/2026 - Lista de Inscritos, formato, pdf, 398kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2864548_sei_2863010_edital_minuta__.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4590,20 +4586,24 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
+          <t>Edital PAEP nº 06/2022 - formato, pdf, 331kb</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/02022022_Edital_1626836_SEI_CAPES___1626182___Edita_6.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F149" t="n">
-        <v>1</v>
-      </c>
-      <c r="G149" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Alteração do Edital PAEP nº 06/2022 - formato, pdf, 80kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15062022_Edital_1733665_Edital_6_2022.pdf/@@display-file/file ; Reabertura do Edital PAEP nº 06/2022 - formato, pdf, 112kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/24032022_Edital_1661092_Edital_6.2022_reabertura.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4613,20 +4613,24 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
+          <t>Edital PAEP nº 11/2023 - formato, pdf, 264kb</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20042023_Edital_1959492_SEI_CAPES___1959158___Edital_11_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F150" t="n">
-        <v>1</v>
-      </c>
-      <c r="G150" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Alteração doEdital PAEP nº 11/2023 - formato, pdf, 154kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08092023_EDITAL112023ALTERAO.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4636,22 +4640,22 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
+          <t>Edital PAEP nº 19/2025 - formato, pdf, 136kb</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12092025_Edital_2679718_SEI_2669828_Edital_19_2025.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F151" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
+          <t>Alteração do edital PAEP nº 19/2025 - formato, pdf, 51kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23102025_Edital_2706985_SEI_2706736_Edital_n__19_2025___ALTERACAO.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4663,22 +4667,22 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
+          <t>Edital PAEP nº 22/2024 - Alteração - formato, pdf, 47kb</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="inlineStr"/>
       <c r="E152" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/Edital_2473082_SEI_2472594_Edital_22_2024___ALTERACAO.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F152" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+          <t>Edital PAEP nº 22/2024 - formato, pdf, 126kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/10092024_Edital_2457107_SEI_2457028_Edital_22_2024.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4690,24 +4694,20 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
+          <t>Edital PAEP nº 37/2023 - formato, pdf, 264kb</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="inlineStr"/>
       <c r="E153" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122023_Edital_2295422_SEI_2295394_Edital_37_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F153" t="n">
-        <v>4</v>
-      </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4717,22 +4717,22 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
+          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F154" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
+          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4744,24 +4744,20 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
+          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F155" t="n">
-        <v>3</v>
-      </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4771,14 +4767,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
+          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -4789,134 +4785,154 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
+          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F157" t="n">
-        <v>1</v>
-      </c>
-      <c r="G157" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
+          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F158" t="n">
-        <v>1</v>
-      </c>
-      <c r="G158" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
+          <t>Lista de instituições e cursos pré-aprovados para a 3ª fase do Edital nº 08/2022 - Parfor - formato, pdf, 715kb</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/06052022_Relacao_1700579_LISTA_DE_IES_E_CURSOS_APROVADOS_PARA_A_3__ETAPA_DO_EDITAL_CAPES_N__08.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F159" t="n">
-        <v>1</v>
-      </c>
-      <c r="G159" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Alteraçãodo Edital nº 08/2022 - Parfor - formato, xls, 119kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/20122022_Edital_1880841_Edital_8_2022___PARFOR.pdf/@@display-file/file ; Alteração do Edital nº 08/2022 - Parfor - formato, pdf, 128kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09062022_Edital_1729649_EDITAL___8_2022.pdf/@@display-file/file ; Edital nº 08/2022 - Parfor - formato, pdf, 203kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/07022022_Edital_1629612_SEI_CAPES___1628279___Edital_8.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
+          <t>Lista e inscritos do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 520kb</t>
         </is>
       </c>
       <c r="C160" t="inlineStr"/>
       <c r="D160" t="inlineStr"/>
       <c r="E160" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/20022024_Lista_Listagem_2324280_SEI_2323841_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F160" t="n">
-        <v>1</v>
-      </c>
-      <c r="G160" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Alteração do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/12062024_Edital_2395239_SEI_2389783_Edital_34_2023.pdf/@@display-file/file ; Prorrogação do Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 54kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/28122023_Edital_2301024_SEI_2300438_Edital_Conjunto_n__34_2023_Prorrogacao.pdf/@@display-file/file ; Edital nº 34/2023 - Programa Caminhos Amefricanos, formato, pdf, 129kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/04122024_Edital_2282364_SEI_2279471_Edital_Conjunto_n__34_2023.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
+          <t>Lista final de inscritos no Edital n° 33/2022 - Brafitec, formato, pdf, 372kb</t>
         </is>
       </c>
       <c r="C161" t="inlineStr"/>
       <c r="D161" t="inlineStr"/>
       <c r="E161" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/22092022_Lista_Listagem_1808291_Lista_inscritos_Brafitec_Edital_33_22.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F161" t="n">
-        <v>1</v>
-      </c>
-      <c r="G161" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Alteração do Edital n° 33/2022 - Brafitec, formato, pdf, 193kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/23022023_Edital_1920292_Edital_33_22.pdf/@@display-file/file ; Edital n° 33/2022 - Brafitec, formato, pdf, 428kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29062022_EDITAL33_2022_BRAFITEC.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SETEC</t>
+          <t>CAPES</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
+          <t>Prorrogação do Edital nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 69kb</t>
         </is>
       </c>
       <c r="C162" t="inlineStr"/>
       <c r="D162" t="inlineStr"/>
       <c r="E162" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/30082024_Edital_2450719_SEI_2446271_Edital_Conjunto_1_2024.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F162" t="n">
@@ -4932,14 +4948,14 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade</t>
         </is>
       </c>
       <c r="C163" t="inlineStr"/>
       <c r="D163" t="inlineStr"/>
       <c r="E163" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F163" t="n">
@@ -4955,14 +4971,14 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
+          <t>Chamada (documento Nº 6991254) para seleção de unidades da Rede Federal de Educação Profissional e Tecnológica e das redes públicas estaduais de Educação Profissional e Tecnológica, interessadas em receber apoio técnico para a implementação de programas de aprendizagem profissional articulados a cursos técnicos ou de qualificação profissional com componentes curriculares relacionados à sustentabilidade.</t>
         </is>
       </c>
       <c r="C164" t="inlineStr"/>
       <c r="D164" t="inlineStr"/>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/SEI_6991254_chamada.pdf</t>
         </is>
       </c>
       <c r="F164" t="n">
@@ -4978,14 +4994,14 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
+          <t>Chamada Pública com o objetivo de identificar, avaliar, cadastrar e disponibilizar metodologias, ferramentas e estudos sobre o mapeamento de demandas por Educação Profissional Técnica de Nível Médio, visando aprimorar a definição de ofertas de Educação Profissional Técnica de Nível Médio, no âmbito do Programa Juros por Educação.</t>
         </is>
       </c>
       <c r="C165" t="inlineStr"/>
       <c r="D165" t="inlineStr"/>
       <c r="E165" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/SEI_6268868_Resultado_de_Edital.pdf</t>
         </is>
       </c>
       <c r="F165" t="n">
@@ -5001,14 +5017,14 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
+          <t>Chamada Pública de Adesão das Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT), com objetivo de capacitação técnica para submissão de propostas em futuros editais de unidades Embrapii.</t>
         </is>
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="inlineStr"/>
       <c r="E166" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/edital-2025/SEI_MEC5650163ResultadodeEdital_.pdf</t>
         </is>
       </c>
       <c r="F166" t="n">
@@ -5024,14 +5040,14 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
+          <t>Chamada Pública de Adesão à linha de fomento Qualifica Mais EnergIFE</t>
         </is>
       </c>
       <c r="C167" t="inlineStr"/>
       <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/chamadapublica.pdf</t>
         </is>
       </c>
       <c r="F167" t="n">
@@ -5047,14 +5063,14 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
+          <t>Chamada Pública nº 01/2017 - Trata-se de chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para capacitação em Gestão da Inovação.</t>
         </is>
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr"/>
       <c r="E168" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/extrato_chamada_dou_cp_01_2017.pdf</t>
         </is>
       </c>
       <c r="F168" t="n">
@@ -5070,14 +5086,14 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Chamada Pública nº 01/2018 - Trata-se da chamada pública para seleção de propostas e servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) em efetivo exercício, para participarem da capacitação em Gestão da Inovação (GI - CSIRO).</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="inlineStr"/>
       <c r="E169" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/20181030Edital012018ChamadaPblicaGICSIRO.pdf</t>
         </is>
       </c>
       <c r="F169" t="n">
@@ -5093,14 +5109,14 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
+          <t>Chamada Pública nº 02/2017 - Trata-se de chamada pública para concurso sobre educação profissional da Secretaria de Educação Profissional e Tecnológica (Setec/MEC) em parceria com a Comunidade dos Países de Língua Portuguesa (CPLP).</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="inlineStr"/>
       <c r="E170" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_concurso_cplp_2017.pdf</t>
         </is>
       </c>
       <c r="F170" t="n">
@@ -5116,14 +5132,14 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
+          <t>Chamada Pública nº 02/2018 - Trata-se da chamada pública para seleção de servidores da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) para a capacitação Brasileiros Formando Formadores (BraFF).</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="inlineStr"/>
       <c r="E171" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Edital_02_2018_BRAFF.pdf</t>
         </is>
       </c>
       <c r="F171" t="n">
@@ -5139,14 +5155,14 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
+          <t>Chamada Pública nº 38/2018 - Trata do processo de seleção de propostas para credenciamento de instituições da Rede Federal, Faculdades de Tecnologia do Estado de São Paulo (Fatecs) e do Instituto Tecnológico de Aeronáutica (ITA) para atuação como Núcleo de Línguas (NucLi-IsF) no âmbito do Programa Idiomas sem Fronteiras (IsF).</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2018/Editaln382018ChamadaPblicaparacredenciamentodeinstituiesdaRFEPCTdasFatecsedoITA.pdf</t>
         </is>
       </c>
       <c r="F172" t="n">
@@ -5162,14 +5178,14 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
+          <t>Chamada Pública nº 79/2016 - Trata-se de chamada pública para apresentação de propostas por instituição de educação profissional e tecnológica para a oferta de cursos de formação inicial e continuada ou de qualificação profissional e cursos técnicos de nível médio, presenciais ou à distância, sem transferência de recursos, no âmbito do PRONATEC, denominada “PROPOSTAS VOLUNTÁRIAS - PRONATEC”</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/extrato_edital_79_2016_setec.pdf</t>
         </is>
       </c>
       <c r="F173" t="n">
@@ -5185,14 +5201,14 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
+          <t>Chamada Pública que estabelece os procedimentos para a autorização de oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior (IPES) para fins de habilitação ao Programa Juros por Educação, no âmbito do Programa de Pleno Pagamento de Dívidas dos Estados (Propag).</t>
         </is>
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/FAQEdital6.2025.pdf</t>
         </is>
       </c>
       <c r="F174" t="n">
@@ -5208,14 +5224,14 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
+          <t>Chamamento Público para credenciamento de profissionais no Banco de Especialistas para atuar no Projeto Assistec Inova, junto ao Ministério da Educação, no âmbito da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_23000.035944_2024_89.pdf</t>
         </is>
       </c>
       <c r="F175" t="n">
@@ -5231,14 +5247,14 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
+          <t>Edital 1/2026 - Chamada Pública de Adesão dos Institutos Federais de Educação, Ciência e Tecnologia, do Centro Federal de Educação Tecnológica Celso Suckow da Fonseca, do Centro Federal de Educação Tecnológica de Minas Gerais e do Colégio Pedro II, com objetivo de capacitação técnica para submissão de propostas em futuros editais de Unidades Embrapii.</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/edital12026.pdf</t>
         </is>
       </c>
       <c r="F176" t="n">
@@ -5254,14 +5270,14 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital 84/2021 - Seleção de Projetos para desenvolvimento dos Ambientes de Promotores de Inovação na Rede Federal</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="inlineStr"/>
       <c r="E177" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/ResultadoetapaI.pdf</t>
         </is>
       </c>
       <c r="F177" t="n">
@@ -5277,14 +5293,14 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
+          <t>Edital nº 01/2017 - APRESENTAÇÃO DE PROPOSTAS PARA A OFERTA DE VAGAS GRATUITAS EM CURSOS TÉCNICOS NA FORMA CONCOMITANTE, NO ÂMBITO DO PRONATEC/MEDIOTEC – 2º/2017 - A Secretária de Educação Profissional e Tecnológica do Ministério da Educação, no uso da atribuição que lhe confere o art. 13, Anexo I, do Decreto n° 7.690, de 02 de março de 2012, e considerando o disposto na Lei nº 12.513, de 26 de outubro de 2011, a Portaria nº 817, de 13 de agosto de 2015, a Portaria nº160, de 05 de março de 2013, alterada pela Portaria nº 701, de 13 de agosto de 2014, TORNA PÚBLICO os procedimentos e o cronograma para a apresentação de propostas visando a oferta de vagas gratuitas em cursos técnicos na forma concomitante e na modalidade presencial, no âmbito do Programa Nacional de Acesso ao Ensino Técnico e Emprego - PRONATEC, por meio da ação MEDIOTEC, para ingresso no segundo semestre de 2017.</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="inlineStr"/>
       <c r="E178" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2017/edital_01_mediotec_2017.pdf</t>
         </is>
       </c>
       <c r="F178" t="n">
@@ -5300,14 +5316,14 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
+          <t>Edital nº 08/2024 - Chamamento Público visando à seleção de autores(as) para elaboração de capítulos de obra a ser publicada cuja temática central é a gestão de Núcleos de Inovação Tecnológica (NITs) e/ou de Agências de Inovação da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT) Divulgação das Inscrições Homologadas</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/436.SEI_MEC5030251Edital.pdf</t>
         </is>
       </c>
       <c r="F179" t="n">
@@ -5323,14 +5339,14 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 1/2023 - Seleção de proposta de selo comemorativo, em alusão aos 15 anos dos Institutos Federais.</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
       <c r="E180" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4094376Edital.pdf</t>
         </is>
       </c>
       <c r="F180" t="n">
@@ -5346,14 +5362,14 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
+          <t>Edital nº 100/2022 - Chamamento Público para a seleção de propostas para o Desafio Soutec</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="inlineStr"/>
       <c r="E181" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/editais-2022/SEI_MEC3570188Edital.pdf</t>
         </is>
       </c>
       <c r="F181" t="n">
@@ -5369,14 +5385,14 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Edital nº 26 versão consolidada</t>
+          <t>Edital nº 109/2022 - Chamamento Público - Seleção de projetos voltados à promoção do empreendedorismo inovador, com foco na Economia 4.0, associados ao ensino, à pesquisa e à extensão, destinado às instituições integrantes da Rede Federal de Educação Profissional, Científica e Tecnológica</t>
         </is>
       </c>
       <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr"/>
       <c r="E182" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital109.pdf</t>
         </is>
       </c>
       <c r="F182" t="n">
@@ -5392,14 +5408,14 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 11/2024 - Chamamento Público para a seleção de projetos aptos a integrarem a 4ª Semana Nacional de Educação Profissional e Tecnológica Retificação do</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
       <c r="D183" t="inlineStr"/>
       <c r="E183" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024-1/Edital_11.pdf</t>
         </is>
       </c>
       <c r="F183" t="n">
@@ -5415,24 +5431,20 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
+          <t>Edital nº 15/2023 - Chamada Pública para o Workshop para elaboração de Itinerários Formativos em economia circular na Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C184" t="inlineStr"/>
       <c r="D184" t="inlineStr"/>
       <c r="E184" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_MEC3884064Edital.pdf</t>
         </is>
       </c>
       <c r="F184" t="n">
-        <v>2</v>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -5442,14 +5454,14 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
+          <t>Edital nº 2/2020 - IFES, de chamada pública para a seleção de projetos voltados à implementação das Oficinas 4.0, aberto às autarquias da Rede Federal.</t>
         </is>
       </c>
       <c r="C185" t="inlineStr"/>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19329-chamada-publica-2-2020-apoio-a-implementacao-de-oficinas-4-0</t>
         </is>
       </c>
       <c r="F185" t="n">
@@ -5465,14 +5477,14 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
+          <t>Edital nº 20/2021 – Seleção de servidores para atuação em Projetos de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="inlineStr"/>
       <c r="E186" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/SEI_MEC2573324Edital.pdf</t>
         </is>
       </c>
       <c r="F186" t="n">
@@ -5488,14 +5500,14 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
+          <t>Edital nº 25/2023 - Chamada Pública destinada a selecionar equipes da Rede Federal de Educação Profissional, Científica e Tecnológica (EPCT) para participação no projeto de formação em criatividade, inovação e prototipagem do mercosul (Hackathon Mercosul). Retificação do Edital</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="inlineStr"/>
       <c r="E187" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/SEI_MEC3913111Edital.pdf</t>
         </is>
       </c>
       <c r="F187" t="n">
@@ -5511,14 +5523,14 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
+          <t>Edital nº 26 versão consolidada</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC3980995Documento.pdf</t>
         </is>
       </c>
       <c r="F188" t="n">
@@ -5534,14 +5546,14 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
+          <t>Edital nº 3/2021 – Chamada Pública para seleção de projetos de iniciação tecnológica com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="inlineStr"/>
       <c r="E189" t="inlineStr">
         <is>
-          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19351-chamada-publica-3-2020-projetos-iniciacao-tecnologica-economia-4-0</t>
         </is>
       </c>
       <c r="F189" t="n">
@@ -5557,20 +5569,24 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
+          <t>Edital nº 35/2020 - Chamada Pública - que tem como objetivo selecionar projetos voltados à criação de Laboratórios IFMaker junto aos Institutos Federais de Educação, Ciência e Tecnologia; Centros Federais de Educação Tecnológica Celso Suckow da Fonseca – Cefet-RJ e de Minas Gerais – Cefet-MG e o Colégio Pedro II, conforme especificado no Despacho SEI nº 2064854</t>
         </is>
       </c>
       <c r="C190" t="inlineStr"/>
       <c r="D190" t="inlineStr"/>
       <c r="E190" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/SEI_MEC_2064339_Edital_Chamada_Publica.pdf</t>
         </is>
       </c>
       <c r="F190" t="n">
-        <v>1</v>
-      </c>
-      <c r="G190" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Retificação Edital nº 35/2020 - Chamada Pública - Seleção de projetos voltados à criação de Laboratórios Maker junto à Rede Federal de Educação Profissional, Científica e Tecnológica Retificação de Cronograma ​do | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/AlteraodecronogramaRedeMakeredital35.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -5580,14 +5596,14 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
+          <t>Edital nº 46, de 20 de julho de 2020, que torna público edital para adesão de estados e Distrito Federal à oferta de Curso de Especialização Lato Sensu em Docência para a Educação Profissional e Tecnológica (DocentEPT) aos professores da rede pública estadual e distrital que atuam na oferta de cursos de Educação Profissional e Tecnológica</t>
         </is>
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2020/Editaldeadeso_DOU.pdf</t>
         </is>
       </c>
       <c r="F191" t="n">
@@ -5603,14 +5619,14 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
+          <t>Edital nº 47/2022 - Chamada Pública para oferta de cursos da Plataforma Aprenda Mais</t>
         </is>
       </c>
       <c r="C192" t="inlineStr"/>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln47.pdf</t>
         </is>
       </c>
       <c r="F192" t="n">
@@ -5626,14 +5642,14 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
+          <t>Edital nº 48/2022 - Procedimentos para autorização da oferta de cursos técnicos de nível médio por Instituições Privadas de Ensino Superior – Anexos do</t>
         </is>
       </c>
       <c r="C193" t="inlineStr"/>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2022/Editaln48.pdf</t>
         </is>
       </c>
       <c r="F193" t="n">
@@ -5649,14 +5665,14 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
+          <t>Edital nº 5 /2026 - Seleção de propostas de projetos de extensão voltados ao Acesso, à Permanência e ao Êxito no âmbito da Rede Federal de Educação Profissional, Científica e Tecnológica (RFEPCT).</t>
         </is>
       </c>
       <c r="C194" t="inlineStr"/>
       <c r="D194" t="inlineStr"/>
       <c r="E194" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2026/sei_7012727_edital_5.pdf</t>
         </is>
       </c>
       <c r="F194" t="n">
@@ -5672,14 +5688,14 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
+          <t>Edital nº 5/2020 – Chamada para seleção de projetos de apoio ao empreendedorismo inovador com foco na Economia 4.0. Acesse o edital .</t>
         </is>
       </c>
       <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr"/>
       <c r="E195" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
+          <t>https://www.ifes.edu.br/chamadas-publicas/19384-chamada-publica-05-2020-selecao-de-projetos-de-apoio-ao-empreendedorismo-inovador-com-foco-na-economia-4-0</t>
         </is>
       </c>
       <c r="F195" t="n">
@@ -5695,14 +5711,14 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
+          <t>Edital nº 5/2021 – IF Mais Empreendedor Nacional : Adesão ao Programa IF Mais Empreendedor Nacional</t>
         </is>
       </c>
       <c r="C196" t="inlineStr"/>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital05.2021IFEMPREENDEDORNACIONAL.pdf</t>
         </is>
       </c>
       <c r="F196" t="n">
@@ -5718,14 +5734,14 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
+          <t>Edital nº 5/2024 - Seleção de propostas de novos Cursos Abertos, On-line e Massivos (MOOCs), desenvolvidos pela Rede Federa de Educação Profissional, Científica e Tecnológica, a serem disponibilizados na Plataforma APRENDA MAIS.</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/edital-2023/SEI_MEC4659481Edital.pdf</t>
         </is>
       </c>
       <c r="F197" t="n">
@@ -5741,14 +5757,14 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
+          <t>Edital nº 52/2016 – que torna público, para conhecimento dos interessados, que será realizado na modalidade concurso, o PROJETO DESAFIO DA EDUCAÇÃO PROFISSIONAL E TECNOLÓGICA, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional para aprimorar a Educação Profissional e Tecnológica estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações.</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
       <c r="D198" t="inlineStr"/>
       <c r="E198" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/edital_n_52_2016.pdf</t>
         </is>
       </c>
       <c r="F198" t="n">
@@ -5764,14 +5780,14 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
+          <t>Edital nº 55/2016 , que torna público concurso PROJETO DESAFIO EDUCAÇÃO ZIKAZERO, na forma do REGULAMENTO anexo a este edital, com o objetivo de promover uma campanha nacional de mobilização para o enfrentamento ao Aedes aegyp e à microcefalia estimulando a sociedade a enviar propostas de ações inovadoras e compartilhar experiências exitosas de implementação de ações em prol do combate ao mosquito.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="inlineStr"/>
       <c r="E199" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2016/Edital_55_2016_SEI_MEC_0227936.pdf</t>
         </is>
       </c>
       <c r="F199" t="n">
@@ -5787,14 +5803,14 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
+          <t>Edital nº 6/2021 - Edital de Adesão das instituições ao Sistema Re-Saber</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="inlineStr"/>
       <c r="E200" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/Edital_06_2021.pdf</t>
         </is>
       </c>
       <c r="F200" t="n">
@@ -5810,14 +5826,14 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
+          <t>Edital nº 6/2024 - Edital visa selecionar a proposta de selo/logomarca que será utilizado em confecções comemorativas no contexto dos 115 anos da Rede Federal de Educação Profissional, Científica e Tecnológica, que poderá ser personalizado como selo postal, via Correios. *</t>
         </is>
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="inlineStr"/>
       <c r="E201" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-2024/325.SEI_MEC4985249Edital.pdf</t>
         </is>
       </c>
       <c r="F201" t="n">
@@ -5833,14 +5849,14 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
+          <t>Edital nº 61/2019 – Regulamento do Cadastro de Especialistas para compor o Banco de Avaliadores da Secretaria de Educação Profissional e Tecnológica.</t>
         </is>
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN612019.pdf</t>
         </is>
       </c>
       <c r="F202" t="n">
@@ -5856,14 +5872,14 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+          <t>Edital nº 63/2021- Seleção de Projetos de Promoção às Indicações Geográficas</t>
         </is>
       </c>
       <c r="C203" t="inlineStr"/>
       <c r="D203" t="inlineStr"/>
       <c r="E203" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/editais/2021/Edital63.pdf</t>
         </is>
       </c>
       <c r="F203" t="n">
@@ -5879,14 +5895,14 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+          <t>Edital nº 67/2021 - Chamada Pública de Projetos para apoio à implementação das Oficinas 4.0</t>
         </is>
       </c>
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="inlineStr"/>
       <c r="E204" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/SEI_MEC2898796Edital67.pdf</t>
         </is>
       </c>
       <c r="F204" t="n">
@@ -5902,24 +5918,20 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+          <t>Edital nº 68/2019 – Seleção de servidores para atuação em Projetos Educacionais de Colaboração Técnica junto ao Ministério da Educação.</t>
         </is>
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="inlineStr"/>
       <c r="E205" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2019/EDITALN682019.pdf</t>
         </is>
       </c>
       <c r="F205" t="n">
-        <v>2</v>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -5929,14 +5941,14 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+          <t>Edital nº 83/2022 – Seleção de propostas de instituições da Rede Federal para a implementação de programa de capacitação de estudantes denominado Oficinas 4.0</t>
         </is>
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="inlineStr"/>
       <c r="E206" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital83.2022.pdf</t>
         </is>
       </c>
       <c r="F206" t="n">
@@ -5952,14 +5964,14 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+          <t>Edital nº 88/2022 – Seleção de projetos de iniciação tecnológica de instituições da RFEPCT para o desenvolvimento de ações de formação em programação e/ou robótica e/ou cultura maker para estudantes dos anos finais do ensino fundamental (6º ao 9º ano) das redes públicas de ensino. Retificação ​do</t>
         </is>
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="inlineStr"/>
       <c r="E207" t="inlineStr">
         <is>
-          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Edital88.2022.pdf</t>
         </is>
       </c>
       <c r="F207" t="n">
@@ -5975,20 +5987,162 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+          <t>Edital nº 94/2022 – Chamada Pública para a capacitação de multiplicadores em bioeconomia para a Amazônia Legal. Chamada Pública para a Adesão de parceiros ofertantes da Rede Federal de Educação Profissional, Científica e Tecnológica – RFEPCT à linha de fomento Qualifica Mais EnergIFE, voltada à promoção da oferta de cursos na área das Energias Renováveis. Retificação do</t>
         </is>
       </c>
       <c r="C208" t="inlineStr"/>
       <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr">
         <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Editaln94.2022.pdf</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>1</v>
+      </c>
+      <c r="G208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Edital nº 99/2022 - Chamamento Público para a seleção de projetos de inovação e trabalhos acadêmicos aptos a integrarem a Semana Nacional da Educação Profissional e Tecnológica Retificação do</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr"/>
+      <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/secretarias/secretaria-de-educacao-profissional/SEI_MEC3566713Edital.pdf</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>1</v>
+      </c>
+      <c r="G209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Programa Setec-Capes/NOVA de capacitação para Professores da Rede Federal de Educação Profissional, Científica e Tecnológica . A Secretaria de Educação Profissional e Tecnológica (Setec) do Ministério da Educação, com apoio da Coordenação de Aperfeiçoamento de Pessoal de Nível Superior (Capes), lançam chamada pública de capacitação para professores de inglês em efetivo exercício na Rede Federal de Educação Profissional - Institutos Federais, Cefets, Escolas Técnicas vinculas às Universidades Federais e Colégio Pedro II. (Retificação publicada no Diário Oficial da União em 02 de junho de 2016)</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr"/>
+      <c r="D210" t="inlineStr"/>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/media/seb-1/pdf/editais/2015/chamada_setec_capes_nova_extrato_dou.pdf</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>1</v>
+      </c>
+      <c r="G210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Republicação do Edital nº 76/2022 - Chamamento Público para seleção de projetos voltados ao fortalecimento de Núcleos de Inovação Tecnológica e/ou Agências de Inovação.</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr"/>
+      <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/Republicaodoedital76.pdf</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>2</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Retificação do Edital nº 76/2022 – novo cronograma | https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais-1/editais-2022/SEI_23000.006585_2022_91.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições da Rede Federal de Educação Profissional, Científica e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr"/>
+      <c r="D212" t="inlineStr"/>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital10.pdf</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>1</v>
+      </c>
+      <c r="G212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Privadas de Ensino Superior que ofertam cursos técnicos e Escolas Técnicas Privadas).</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr"/>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/ResultadoEdital09.pdf</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>1</v>
+      </c>
+      <c r="G213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>SETEC</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Seleção de projetos para Mostra Tecnológica da 5ª Semana Nacional da Educação Profissional e Tecnológica (Instituições Públicas Estaduais e Distrital de Educação Profissional e Tecnológica).</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr"/>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr">
+        <is>
           <t>https://www.gov.br/mec/pt-br/acesso-a-informacao/institucional/estrutura-organizacional/orgaos-especificos-singulares/secretaria-de-educacao-profissional/editais/2025/2147-resultado-preliminar.pdf</t>
         </is>
       </c>
-      <c r="F208" t="n">
-        <v>1</v>
-      </c>
-      <c r="G208" t="inlineStr"/>
+      <c r="F214" t="n">
+        <v>1</v>
+      </c>
+      <c r="G214" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: crawl 2026-08-29 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -3108,7 +3108,11 @@
           <t>07/08/2024</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr">
         <is>
           <t>https://www.finep.gov.br/e/chamada-publica/222684/749717</t>

</xml_diff>

<commit_message>
chore: crawl 2026-09-01 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -1529,11 +1529,11 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Prorrogação - Edital Conjunto nº 4/2026, formato, pdf, 52,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/edital_2863852_sei_2863595_edital_conjunto_n__4_2026___prorrogacao.pdf/@@display-file/file</t>
+          <t>Prorrogação - Edital Conjunto nº 4/2026, formato, pdf, 52,5kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/edital_2863852_sei_2863595_edital_conjunto_n__4_2026___prorrogacao.pdf/@@display-file/file ; Alteração - Edital Conjunto nº 4/2026, formato, pdf, 52,6kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/edital_2888100_sei_2886868_edital_conjunto_n__4_2026___alteracao.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4721,22 +4721,22 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
+          <t>Edital PDSE nº 17/2025 – segunda chamada – relação de aprovadas na análise técnica após a análise dos recursos - formato, pdf, 1,438kb</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="inlineStr"/>
       <c r="E154" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/lista_listagem_2878471_listagem_resultado_final_pdse_segunda_chamada.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F154" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>
@@ -4748,20 +4748,24 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
+          <t>Lista de inscritos do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 407kb</t>
         </is>
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/15052024_Lista_Listagem_2374115_Inscritos_MIR.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F155" t="n">
-        <v>1</v>
-      </c>
-      <c r="G155" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Alteração do Edital Conjunto nº 01/2024 - Programa Caminhos Amefricanos, formato, pdf, 63kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/29042024_Edital_2368101_SEI_2365347_Edital_Conjunto_n__1_CAPES_MIR.pdf/@@display-file/file</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4771,14 +4775,14 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
+          <t>Lista de inscritos do Edital nº 05/2024 - Programa CAPES/CLIMAT-AMSUD, formato - pdf, 46kb</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/10062024_Lista_Listagem_2390159_Lista_de_Inscritos_3.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F156" t="n">
@@ -4794,24 +4798,20 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
+          <t>Lista de inscritos doEdital nº 8/202 - CAPES/COFECUB, formato, pdf, 581kb</t>
         </is>
       </c>
       <c r="C157" t="inlineStr"/>
       <c r="D157" t="inlineStr"/>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/14062023_Lista_Listagem_1990268_Inscricoes_cofecub_2023.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F157" t="n">
-        <v>4</v>
-      </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4821,14 +4821,14 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Primeira chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 8,8mb</t>
+          <t>Lista de inscrições - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 393kb</t>
         </is>
       </c>
       <c r="C158" t="inlineStr"/>
       <c r="D158" t="inlineStr"/>
       <c r="E158" t="inlineStr">
         <is>
-          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/29102025_Lista_Listagem_2708089_PDSE.pdf/@@display-file/file</t>
+          <t>https://www.gov.br/capes/pt-br/centrais-de-conteudo/Lista_de_Inscricoes_Homologadas_PDSE___2020_REVISADA.pdf/@@display-file/file</t>
         </is>
       </c>
       <c r="F158" t="n">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Lista de inscrições do Edital nº 17/2025 - Segunda chamada Programa Institucional de Doutorado Sanduíche no Exterior (PDSE) - formato, pdf, 1,4mb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/resultados-dos-editais/27042026_Lista_Listagem_2808119_Lista_de_inscricoes_homologadas_do_Edital_172025___PDSE___segunda_chamada___formato_pdf__2_.pdf/@@display-file/file ; Alteração do Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE), formato, pdf, 52kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/08102025_Edital_2696973_SEI_2695934_Edital_17_2025__.pdf/@@display-file/file ; Edital nº 17/2025 - Programa Institucional de Doutorado Sanduíche no Exterior (PDSE)- formato, pdf, 142kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/21082025_Edital_2662823_SEI_2661209_Edital_n__17_2025.pdf/@@display-file/file</t>
+          <t>Lista de candidaturas - Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 417kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/documentos/diretoria-de-relacoes-internacionais/pdse/Lista_Listagem_1439062_Lista_de_Inscricoes_Homologadas_PDSE___2020.pdf/@@display-file/file ; Retificação do Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE) - formato, pdf, 244kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/EDITAL192020_PDSERETIFICAO.pdf/@@display-file/file ; Edital nº 19/2020 - Programa Doutorado-sanduíche no Exterior (PDSE)- formato, pdf, 236kb | https://www.gov.br/capes/pt-br/centrais-de-conteudo/editais/09102020_edital-19-pdse.pdf/@@display-file/file</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: crawl 2026-09-05 — atualização de editais
</commit_message>
<xml_diff>
--- a/editais.xlsx
+++ b/editais.xlsx
@@ -1282,7 +1282,11 @@
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>08/09/2026</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
           <t>https://www.fapesb.ba.gov.br/diretrizes-especificas-da-fapesb-chamada-mobility-confap-italy-2026/</t>

</xml_diff>